<commit_message>
chore(data-release): publish site data 2026-10-16 14:16:17 UTC
</commit_message>
<xml_diff>
--- a/countries/br-ac/2000-2004.xlsx
+++ b/countries/br-ac/2000-2004.xlsx
@@ -1702,7 +1702,7 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr">
@@ -2792,7 +2792,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK15" t="inlineStr">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK32" t="inlineStr">
@@ -6382,7 +6382,7 @@
       </c>
       <c r="AJ39" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK39" t="inlineStr">
@@ -7472,7 +7472,7 @@
       </c>
       <c r="AJ46" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK46" t="inlineStr">
@@ -11100,7 +11100,7 @@
       </c>
       <c r="AJ71" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK71" t="inlineStr">
@@ -13459,7 +13459,7 @@
       </c>
       <c r="AJ87" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK87" t="inlineStr">
@@ -16100,7 +16100,7 @@
       </c>
       <c r="AJ105" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK105" t="inlineStr">
@@ -18741,7 +18741,7 @@
       </c>
       <c r="AJ123" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK123" t="inlineStr">
@@ -20254,7 +20254,7 @@
       </c>
       <c r="AJ133" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK133" t="inlineStr">
@@ -24023,7 +24023,7 @@
       </c>
       <c r="AJ159" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK159" t="inlineStr">
@@ -27792,7 +27792,7 @@
       </c>
       <c r="AJ185" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK185" t="inlineStr">
@@ -29305,7 +29305,7 @@
       </c>
       <c r="AJ195" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK195" t="inlineStr">
@@ -34202,7 +34202,7 @@
       </c>
       <c r="AJ229" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK229" t="inlineStr">
@@ -42483,7 +42483,7 @@
       </c>
       <c r="AJ287" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK287" t="inlineStr">
@@ -49636,7 +49636,7 @@
       </c>
       <c r="AJ337" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK337" t="inlineStr">
@@ -54533,7 +54533,7 @@
       </c>
       <c r="AJ371" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK371" t="inlineStr">
@@ -59712,7 +59712,7 @@
       </c>
       <c r="AJ407" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK407" t="inlineStr">
@@ -61366,7 +61366,7 @@
       </c>
       <c r="AJ418" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK418" t="inlineStr">
@@ -63020,7 +63020,7 @@
       </c>
       <c r="AJ429" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK429" t="inlineStr">
@@ -64674,7 +64674,7 @@
       </c>
       <c r="AJ440" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK440" t="inlineStr">
@@ -67597,7 +67597,7 @@
       </c>
       <c r="AJ460" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK460" t="inlineStr">
@@ -70520,7 +70520,7 @@
       </c>
       <c r="AJ480" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK480" t="inlineStr">
@@ -73443,7 +73443,7 @@
       </c>
       <c r="AJ500" t="inlineStr">
         <is>
-          <t>globalid-disease-ontology:2026.09.26.1</t>
+          <t>globalid-disease-ontology:2026.10.16.1</t>
         </is>
       </c>
       <c r="AK500" t="inlineStr">

</xml_diff>